<commit_message>
Atualização automática de dados local - 30/06/2026 11:10
</commit_message>
<xml_diff>
--- a/planilhas_para_atualizar/EAR_DIARIO_SUBSISTEMA_2026.xlsx
+++ b/planilhas_para_atualizar/EAR_DIARIO_SUBSISTEMA_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="14">
   <si>
     <t>id_subsistema</t>
   </si>
@@ -423,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F705"/>
+  <dimension ref="A1:F717"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -12885,10 +12885,10 @@
         <v>15302.396</v>
       </c>
       <c r="E623" s="3">
-        <v>14885.256</v>
+        <v>14887.174</v>
       </c>
       <c r="F623" s="3">
-        <v>97.274</v>
+        <v>97.28660000000001</v>
       </c>
     </row>
     <row r="624" spans="1:6">
@@ -12965,10 +12965,10 @@
         <v>15302.396</v>
       </c>
       <c r="E627" s="3">
-        <v>14924.187</v>
+        <v>14925.146</v>
       </c>
       <c r="F627" s="3">
-        <v>97.5284</v>
+        <v>97.5347</v>
       </c>
     </row>
     <row r="628" spans="1:6">
@@ -13045,10 +13045,10 @@
         <v>15302.396</v>
       </c>
       <c r="E631" s="3">
-        <v>14946.646</v>
+        <v>14949.524</v>
       </c>
       <c r="F631" s="3">
-        <v>97.6752</v>
+        <v>97.694</v>
       </c>
     </row>
     <row r="632" spans="1:6">
@@ -13125,10 +13125,10 @@
         <v>15302.396</v>
       </c>
       <c r="E635" s="3">
-        <v>14967.87</v>
+        <v>14970.748</v>
       </c>
       <c r="F635" s="3">
-        <v>97.8139</v>
+        <v>97.8327</v>
       </c>
     </row>
     <row r="636" spans="1:6">
@@ -13205,10 +13205,10 @@
         <v>15302.396</v>
       </c>
       <c r="E639" s="3">
-        <v>14954.598</v>
+        <v>14957.476</v>
       </c>
       <c r="F639" s="3">
-        <v>97.7272</v>
+        <v>97.746</v>
       </c>
     </row>
     <row r="640" spans="1:6">
@@ -13285,10 +13285,10 @@
         <v>15302.396</v>
       </c>
       <c r="E643" s="3">
-        <v>14941.371</v>
+        <v>14944.248</v>
       </c>
       <c r="F643" s="3">
-        <v>97.6407</v>
+        <v>97.65949999999999</v>
       </c>
     </row>
     <row r="644" spans="1:6">
@@ -13365,10 +13365,10 @@
         <v>15302.396</v>
       </c>
       <c r="E647" s="3">
-        <v>14923.709</v>
+        <v>14926.585</v>
       </c>
       <c r="F647" s="3">
-        <v>97.5253</v>
+        <v>97.5441</v>
       </c>
     </row>
     <row r="648" spans="1:6">
@@ -13445,10 +13445,10 @@
         <v>15302.396</v>
       </c>
       <c r="E651" s="3">
-        <v>14892.083</v>
+        <v>14896.874</v>
       </c>
       <c r="F651" s="3">
-        <v>97.3186</v>
+        <v>97.34990000000001</v>
       </c>
     </row>
     <row r="652" spans="1:6">
@@ -13525,10 +13525,10 @@
         <v>15302.396</v>
       </c>
       <c r="E655" s="3">
-        <v>14835.362</v>
+        <v>14839.192</v>
       </c>
       <c r="F655" s="3">
-        <v>96.94799999999999</v>
+        <v>96.973</v>
       </c>
     </row>
     <row r="656" spans="1:6">
@@ -13585,10 +13585,10 @@
         <v>51691.226</v>
       </c>
       <c r="E658" s="3">
-        <v>47336.405</v>
+        <v>47333.205</v>
       </c>
       <c r="F658" s="3">
-        <v>91.5753</v>
+        <v>91.56910000000001</v>
       </c>
     </row>
     <row r="659" spans="1:6">
@@ -13605,10 +13605,10 @@
         <v>15302.396</v>
       </c>
       <c r="E659" s="3">
-        <v>14817.83</v>
+        <v>14822.616</v>
       </c>
       <c r="F659" s="3">
-        <v>96.8334</v>
+        <v>96.8647</v>
       </c>
     </row>
     <row r="660" spans="1:6">
@@ -13625,10 +13625,10 @@
         <v>204615.328</v>
       </c>
       <c r="E660" s="3">
-        <v>134507.862</v>
+        <v>134512.204</v>
       </c>
       <c r="F660" s="3">
-        <v>65.73690000000001</v>
+        <v>65.73909999999999</v>
       </c>
     </row>
     <row r="661" spans="1:6">
@@ -13665,10 +13665,10 @@
         <v>51691.226</v>
       </c>
       <c r="E662" s="3">
-        <v>47245.965</v>
+        <v>47241.165</v>
       </c>
       <c r="F662" s="3">
-        <v>91.4004</v>
+        <v>91.39109999999999</v>
       </c>
     </row>
     <row r="663" spans="1:6">
@@ -13685,10 +13685,10 @@
         <v>15302.396</v>
       </c>
       <c r="E663" s="3">
-        <v>14787.87</v>
+        <v>14791.697</v>
       </c>
       <c r="F663" s="3">
-        <v>96.63760000000001</v>
+        <v>96.6626</v>
       </c>
     </row>
     <row r="664" spans="1:6">
@@ -13705,10 +13705,10 @@
         <v>204615.328</v>
       </c>
       <c r="E664" s="3">
-        <v>134629.078</v>
+        <v>134633.366</v>
       </c>
       <c r="F664" s="3">
-        <v>65.7962</v>
+        <v>65.7983</v>
       </c>
     </row>
     <row r="665" spans="1:6">
@@ -13745,10 +13745,10 @@
         <v>51691.226</v>
       </c>
       <c r="E666" s="3">
-        <v>47138.109</v>
+        <v>47133.31</v>
       </c>
       <c r="F666" s="3">
-        <v>91.1917</v>
+        <v>91.1824</v>
       </c>
     </row>
     <row r="667" spans="1:6">
@@ -13765,10 +13765,10 @@
         <v>15302.396</v>
       </c>
       <c r="E667" s="3">
-        <v>14747.035</v>
+        <v>14750.859</v>
       </c>
       <c r="F667" s="3">
-        <v>96.3708</v>
+        <v>96.39570000000001</v>
       </c>
     </row>
     <row r="668" spans="1:6">
@@ -13785,10 +13785,10 @@
         <v>204615.328</v>
       </c>
       <c r="E668" s="3">
-        <v>134635.44</v>
+        <v>134645.375</v>
       </c>
       <c r="F668" s="3">
-        <v>65.7993</v>
+        <v>65.80410000000001</v>
       </c>
     </row>
     <row r="669" spans="1:6">
@@ -13825,10 +13825,10 @@
         <v>51691.226</v>
       </c>
       <c r="E670" s="3">
-        <v>47045.952</v>
+        <v>47037.954</v>
       </c>
       <c r="F670" s="3">
-        <v>91.0134</v>
+        <v>90.9979</v>
       </c>
     </row>
     <row r="671" spans="1:6">
@@ -13845,10 +13845,10 @@
         <v>15302.396</v>
       </c>
       <c r="E671" s="3">
-        <v>14666.604</v>
+        <v>14671.379</v>
       </c>
       <c r="F671" s="3">
-        <v>95.8451</v>
+        <v>95.8764</v>
       </c>
     </row>
     <row r="672" spans="1:6">
@@ -13865,10 +13865,10 @@
         <v>204615.328</v>
       </c>
       <c r="E672" s="3">
-        <v>134600.449</v>
+        <v>134609.003</v>
       </c>
       <c r="F672" s="3">
-        <v>65.7822</v>
+        <v>65.7864</v>
       </c>
     </row>
     <row r="673" spans="1:6">
@@ -13905,10 +13905,10 @@
         <v>51691.226</v>
       </c>
       <c r="E674" s="3">
-        <v>46995.297</v>
+        <v>46945.79</v>
       </c>
       <c r="F674" s="3">
-        <v>90.91540000000001</v>
+        <v>90.81959999999999</v>
       </c>
     </row>
     <row r="675" spans="1:6">
@@ -13925,10 +13925,10 @@
         <v>15302.396</v>
       </c>
       <c r="E675" s="3">
-        <v>14655.876</v>
+        <v>14660.65</v>
       </c>
       <c r="F675" s="3">
-        <v>95.77500000000001</v>
+        <v>95.8062</v>
       </c>
     </row>
     <row r="676" spans="1:6">
@@ -13945,10 +13945,10 @@
         <v>204615.328</v>
       </c>
       <c r="E676" s="3">
-        <v>134652.389</v>
+        <v>134657.769</v>
       </c>
       <c r="F676" s="3">
-        <v>65.80759999999999</v>
+        <v>65.81019999999999</v>
       </c>
     </row>
     <row r="677" spans="1:6">
@@ -13985,10 +13985,10 @@
         <v>51691.226</v>
       </c>
       <c r="E678" s="3">
-        <v>46942.67</v>
+        <v>46846.987</v>
       </c>
       <c r="F678" s="3">
-        <v>90.81359999999999</v>
+        <v>90.6285</v>
       </c>
     </row>
     <row r="679" spans="1:6">
@@ -14005,10 +14005,10 @@
         <v>15302.396</v>
       </c>
       <c r="E679" s="3">
-        <v>14641.478</v>
+        <v>14646.251</v>
       </c>
       <c r="F679" s="3">
-        <v>95.681</v>
+        <v>95.71210000000001</v>
       </c>
     </row>
     <row r="680" spans="1:6">
@@ -14025,10 +14025,10 @@
         <v>204615.328</v>
       </c>
       <c r="E680" s="3">
-        <v>134493.763</v>
+        <v>134496.299</v>
       </c>
       <c r="F680" s="3">
-        <v>65.73009999999999</v>
+        <v>65.7313</v>
       </c>
     </row>
     <row r="681" spans="1:6">
@@ -14065,10 +14065,10 @@
         <v>51691.226</v>
       </c>
       <c r="E682" s="3">
-        <v>46895.597</v>
+        <v>46759.88</v>
       </c>
       <c r="F682" s="3">
-        <v>90.7225</v>
+        <v>90.45999999999999</v>
       </c>
     </row>
     <row r="683" spans="1:6">
@@ -14085,10 +14085,10 @@
         <v>15302.396</v>
       </c>
       <c r="E683" s="3">
-        <v>14603.555</v>
+        <v>14609.085</v>
       </c>
       <c r="F683" s="3">
-        <v>95.4331</v>
+        <v>95.4693</v>
       </c>
     </row>
     <row r="684" spans="1:6">
@@ -14105,10 +14105,10 @@
         <v>204615.328</v>
       </c>
       <c r="E684" s="3">
-        <v>134337.186</v>
+        <v>134340.147</v>
       </c>
       <c r="F684" s="3">
-        <v>65.65349999999999</v>
+        <v>65.655</v>
       </c>
     </row>
     <row r="685" spans="1:6">
@@ -14125,10 +14125,10 @@
         <v>20459.242</v>
       </c>
       <c r="E685" s="3">
-        <v>11412.81</v>
+        <v>11407.127</v>
       </c>
       <c r="F685" s="3">
-        <v>55.7832</v>
+        <v>55.7554</v>
       </c>
     </row>
     <row r="686" spans="1:6">
@@ -14145,10 +14145,10 @@
         <v>51691.226</v>
       </c>
       <c r="E686" s="3">
-        <v>46848.62</v>
+        <v>46708.236</v>
       </c>
       <c r="F686" s="3">
-        <v>90.6317</v>
+        <v>90.3601</v>
       </c>
     </row>
     <row r="687" spans="1:6">
@@ -14165,10 +14165,10 @@
         <v>15302.396</v>
       </c>
       <c r="E687" s="3">
-        <v>14576.355</v>
+        <v>14581.123</v>
       </c>
       <c r="F687" s="3">
-        <v>95.25539999999999</v>
+        <v>95.2865</v>
       </c>
     </row>
     <row r="688" spans="1:6">
@@ -14185,10 +14185,10 @@
         <v>204615.328</v>
       </c>
       <c r="E688" s="3">
-        <v>134332.142</v>
+        <v>134327.066</v>
       </c>
       <c r="F688" s="3">
-        <v>65.6511</v>
+        <v>65.6486</v>
       </c>
     </row>
     <row r="689" spans="1:6">
@@ -14225,10 +14225,10 @@
         <v>51691.226</v>
       </c>
       <c r="E690" s="3">
-        <v>46795.952</v>
+        <v>46653.971</v>
       </c>
       <c r="F690" s="3">
-        <v>90.52979999999999</v>
+        <v>90.2551</v>
       </c>
     </row>
     <row r="691" spans="1:6">
@@ -14245,10 +14245,10 @@
         <v>15302.396</v>
       </c>
       <c r="E691" s="3">
-        <v>14558.172</v>
+        <v>14563.892</v>
       </c>
       <c r="F691" s="3">
-        <v>95.1366</v>
+        <v>95.1739</v>
       </c>
     </row>
     <row r="692" spans="1:6">
@@ -14265,10 +14265,10 @@
         <v>204615.328</v>
       </c>
       <c r="E692" s="3">
-        <v>134104.947</v>
+        <v>134101.601</v>
       </c>
       <c r="F692" s="3">
-        <v>65.54000000000001</v>
+        <v>65.5384</v>
       </c>
     </row>
     <row r="693" spans="1:6">
@@ -14285,10 +14285,10 @@
         <v>20459.242</v>
       </c>
       <c r="E693" s="3">
-        <v>11443.612</v>
+        <v>11445.048</v>
       </c>
       <c r="F693" s="3">
-        <v>55.9337</v>
+        <v>55.9407</v>
       </c>
     </row>
     <row r="694" spans="1:6">
@@ -14305,10 +14305,10 @@
         <v>51691.226</v>
       </c>
       <c r="E694" s="3">
-        <v>46749.027</v>
+        <v>46563.948</v>
       </c>
       <c r="F694" s="3">
-        <v>90.43899999999999</v>
+        <v>90.081</v>
       </c>
     </row>
     <row r="695" spans="1:6">
@@ -14325,10 +14325,10 @@
         <v>15302.396</v>
       </c>
       <c r="E695" s="3">
-        <v>14533.949</v>
+        <v>14541.572</v>
       </c>
       <c r="F695" s="3">
-        <v>94.9783</v>
+        <v>95.02809999999999</v>
       </c>
     </row>
     <row r="696" spans="1:6">
@@ -14345,10 +14345,10 @@
         <v>204615.328</v>
       </c>
       <c r="E696" s="3">
-        <v>134087.423</v>
+        <v>134080.453</v>
       </c>
       <c r="F696" s="3">
-        <v>65.53149999999999</v>
+        <v>65.52809999999999</v>
       </c>
     </row>
     <row r="697" spans="1:6">
@@ -14365,10 +14365,10 @@
         <v>20459.242</v>
       </c>
       <c r="E697" s="3">
-        <v>11544.237</v>
+        <v>11547.081</v>
       </c>
       <c r="F697" s="3">
-        <v>56.4255</v>
+        <v>56.4394</v>
       </c>
     </row>
     <row r="698" spans="1:6">
@@ -14385,10 +14385,10 @@
         <v>51691.226</v>
       </c>
       <c r="E698" s="3">
-        <v>46702.951</v>
+        <v>46509.876</v>
       </c>
       <c r="F698" s="3">
-        <v>90.34990000000001</v>
+        <v>89.97629999999999</v>
       </c>
     </row>
     <row r="699" spans="1:6">
@@ -14405,10 +14405,10 @@
         <v>15302.396</v>
       </c>
       <c r="E699" s="3">
-        <v>14518.849</v>
+        <v>14513.072</v>
       </c>
       <c r="F699" s="3">
-        <v>94.8796</v>
+        <v>94.84180000000001</v>
       </c>
     </row>
     <row r="700" spans="1:6">
@@ -14425,10 +14425,10 @@
         <v>204615.328</v>
       </c>
       <c r="E700" s="3">
-        <v>134236.756</v>
+        <v>134207.491</v>
       </c>
       <c r="F700" s="3">
-        <v>65.6044</v>
+        <v>65.59010000000001</v>
       </c>
     </row>
     <row r="701" spans="1:6">
@@ -14445,10 +14445,10 @@
         <v>20459.242</v>
       </c>
       <c r="E701" s="3">
-        <v>11591.888</v>
+        <v>11587.649</v>
       </c>
       <c r="F701" s="3">
-        <v>56.6584</v>
+        <v>56.6377</v>
       </c>
     </row>
     <row r="702" spans="1:6">
@@ -14465,10 +14465,10 @@
         <v>51691.226</v>
       </c>
       <c r="E702" s="3">
-        <v>46394.417</v>
+        <v>46421.84</v>
       </c>
       <c r="F702" s="3">
-        <v>89.753</v>
+        <v>89.806</v>
       </c>
     </row>
     <row r="703" spans="1:6">
@@ -14485,10 +14485,10 @@
         <v>15302.396</v>
       </c>
       <c r="E703" s="3">
-        <v>14487.027</v>
+        <v>14494.141</v>
       </c>
       <c r="F703" s="3">
-        <v>94.6716</v>
+        <v>94.71810000000001</v>
       </c>
     </row>
     <row r="704" spans="1:6">
@@ -14505,10 +14505,10 @@
         <v>204615.328</v>
       </c>
       <c r="E704" s="3">
-        <v>134231.985</v>
+        <v>134287.291</v>
       </c>
       <c r="F704" s="3">
-        <v>65.60209999999999</v>
+        <v>65.62909999999999</v>
       </c>
     </row>
     <row r="705" spans="1:6">
@@ -14525,10 +14525,250 @@
         <v>20459.242</v>
       </c>
       <c r="E705" s="3">
-        <v>11608.471</v>
+        <v>11608.48</v>
       </c>
       <c r="F705" s="3">
         <v>56.7395</v>
+      </c>
+    </row>
+    <row r="706" spans="1:6">
+      <c r="A706" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B706" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C706" s="5">
+        <v>46199</v>
+      </c>
+      <c r="D706" s="3">
+        <v>51691.226</v>
+      </c>
+      <c r="E706" s="3">
+        <v>46367.647</v>
+      </c>
+      <c r="F706" s="3">
+        <v>89.7012</v>
+      </c>
+    </row>
+    <row r="707" spans="1:6">
+      <c r="A707" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B707" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C707" s="5">
+        <v>46199</v>
+      </c>
+      <c r="D707" s="3">
+        <v>15302.396</v>
+      </c>
+      <c r="E707" s="3">
+        <v>14469.014</v>
+      </c>
+      <c r="F707" s="3">
+        <v>94.5539</v>
+      </c>
+    </row>
+    <row r="708" spans="1:6">
+      <c r="A708" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B708" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C708" s="5">
+        <v>46199</v>
+      </c>
+      <c r="D708" s="3">
+        <v>204615.328</v>
+      </c>
+      <c r="E708" s="3">
+        <v>134259.672</v>
+      </c>
+      <c r="F708" s="3">
+        <v>65.6156</v>
+      </c>
+    </row>
+    <row r="709" spans="1:6">
+      <c r="A709" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B709" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C709" s="5">
+        <v>46199</v>
+      </c>
+      <c r="D709" s="3">
+        <v>20459.242</v>
+      </c>
+      <c r="E709" s="3">
+        <v>11585.81</v>
+      </c>
+      <c r="F709" s="3">
+        <v>56.6287</v>
+      </c>
+    </row>
+    <row r="710" spans="1:6">
+      <c r="A710" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B710" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C710" s="5">
+        <v>46200</v>
+      </c>
+      <c r="D710" s="3">
+        <v>51691.226</v>
+      </c>
+      <c r="E710" s="3">
+        <v>46266.156</v>
+      </c>
+      <c r="F710" s="3">
+        <v>89.50490000000001</v>
+      </c>
+    </row>
+    <row r="711" spans="1:6">
+      <c r="A711" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B711" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C711" s="5">
+        <v>46200</v>
+      </c>
+      <c r="D711" s="3">
+        <v>15302.396</v>
+      </c>
+      <c r="E711" s="3">
+        <v>14433.632</v>
+      </c>
+      <c r="F711" s="3">
+        <v>94.3227</v>
+      </c>
+    </row>
+    <row r="712" spans="1:6">
+      <c r="A712" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B712" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C712" s="5">
+        <v>46200</v>
+      </c>
+      <c r="D712" s="3">
+        <v>204615.328</v>
+      </c>
+      <c r="E712" s="3">
+        <v>134307.169</v>
+      </c>
+      <c r="F712" s="3">
+        <v>65.63890000000001</v>
+      </c>
+    </row>
+    <row r="713" spans="1:6">
+      <c r="A713" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B713" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C713" s="5">
+        <v>46200</v>
+      </c>
+      <c r="D713" s="3">
+        <v>20459.242</v>
+      </c>
+      <c r="E713" s="3">
+        <v>11604.635</v>
+      </c>
+      <c r="F713" s="3">
+        <v>56.7207</v>
+      </c>
+    </row>
+    <row r="714" spans="1:6">
+      <c r="A714" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B714" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C714" s="5">
+        <v>46201</v>
+      </c>
+      <c r="D714" s="3">
+        <v>51691.226</v>
+      </c>
+      <c r="E714" s="3">
+        <v>46173.767</v>
+      </c>
+      <c r="F714" s="3">
+        <v>89.3261</v>
+      </c>
+    </row>
+    <row r="715" spans="1:6">
+      <c r="A715" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B715" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C715" s="5">
+        <v>46201</v>
+      </c>
+      <c r="D715" s="3">
+        <v>15302.396</v>
+      </c>
+      <c r="E715" s="3">
+        <v>14416.698</v>
+      </c>
+      <c r="F715" s="3">
+        <v>94.212</v>
+      </c>
+    </row>
+    <row r="716" spans="1:6">
+      <c r="A716" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B716" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C716" s="5">
+        <v>46201</v>
+      </c>
+      <c r="D716" s="3">
+        <v>204615.328</v>
+      </c>
+      <c r="E716" s="3">
+        <v>134341.945</v>
+      </c>
+      <c r="F716" s="3">
+        <v>65.6559</v>
+      </c>
+    </row>
+    <row r="717" spans="1:6">
+      <c r="A717" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B717" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C717" s="5">
+        <v>46201</v>
+      </c>
+      <c r="D717" s="3">
+        <v>20459.242</v>
+      </c>
+      <c r="E717" s="3">
+        <v>11845.198</v>
+      </c>
+      <c r="F717" s="3">
+        <v>57.8966</v>
       </c>
     </row>
   </sheetData>

</xml_diff>